<commit_message>
Add complete BharatBites manual QA testing project
</commit_message>
<xml_diff>
--- a/05_Test_Cases/BharatBites_Test_Cases.xlsx
+++ b/05_Test_Cases/BharatBites_Test_Cases.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="R8d88e7b5906c461d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="R93e0704f5f18418d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -45,7 +45,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="16">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -79,6 +79,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -299,15 +300,15 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="35" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="35" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="55" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="55" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="38" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="58" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="58" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -604,28 +605,28 @@
         <x:v>BB_TC_009</x:v>
       </x:c>
       <x:c r="B10" s="14" t="str">
-        <x:v>BB_REQ_010</x:v>
+        <x:v>BB_REQ_010; BB_REQ_011</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
-        <x:v>BB_TS_011</x:v>
+        <x:v>BB_TS_011; BB_TS_012; BB_TS_013</x:v>
       </x:c>
       <x:c r="D10" s="14" t="str">
         <x:v>Search</x:v>
       </x:c>
       <x:c r="E10" s="14" t="str">
-        <x:v>Search restaurant/food</x:v>
+        <x:v>Search food items and restaurants with relevant results</x:v>
       </x:c>
       <x:c r="F10" s="14" t="str">
-        <x:v>User is logged in</x:v>
+        <x:v>User is logged in and searchable food/restaurants exist</x:v>
       </x:c>
       <x:c r="G10" s="14" t="str">
-        <x:v>Biryani</x:v>
+        <x:v>Food: Biryani; Restaurant: Spice Garden</x:v>
       </x:c>
       <x:c r="H10" s="14" t="str">
-        <x:v>Enter search term; submit search</x:v>
+        <x:v>Search for Biryani and verify matching food results; search for Spice Garden and verify matching restaurant results</x:v>
       </x:c>
       <x:c r="I10" s="14" t="str">
-        <x:v>Relevant results display</x:v>
+        <x:v>Relevant matching food and restaurant results are displayed</x:v>
       </x:c>
       <x:c r="J10" s="14" t="str">
         <x:v>High</x:v>
@@ -2315,13 +2316,13 @@
         <x:v>Registered account exists</x:v>
       </x:c>
       <x:c r="G63" s="14" t="str">
-        <x:v>Registered email</x:v>
+        <x:v>registereduser@example.com</x:v>
       </x:c>
       <x:c r="H63" s="14" t="str">
-        <x:v>Submit password recovery</x:v>
+        <x:v>Open Forgot Password; enter registered email; submit recovery request</x:v>
       </x:c>
       <x:c r="I63" s="14" t="str">
-        <x:v>Reset instructions are provided</x:v>
+        <x:v>Password reset instructions are provided without exposing sensitive account information</x:v>
       </x:c>
       <x:c r="J63" s="14" t="str">
         <x:v>High</x:v>
@@ -2344,16 +2345,16 @@
         <x:v>Recovery with unregistered email</x:v>
       </x:c>
       <x:c r="F64" s="14" t="str">
-        <x:v>Forgot Password page open</x:v>
+        <x:v>Forgot Password page is open</x:v>
       </x:c>
       <x:c r="G64" s="14" t="str">
         <x:v>notregistered@example.com</x:v>
       </x:c>
       <x:c r="H64" s="14" t="str">
-        <x:v>Submit recovery request</x:v>
+        <x:v>Enter unregistered email; submit recovery request</x:v>
       </x:c>
       <x:c r="I64" s="14" t="str">
-        <x:v>Secure generic response is shown</x:v>
+        <x:v>A secure generic response is shown without confirming whether the account exists</x:v>
       </x:c>
       <x:c r="J64" s="14" t="str">
         <x:v>High</x:v>
@@ -2373,19 +2374,19 @@
         <x:v>Cart</x:v>
       </x:c>
       <x:c r="E65" s="14" t="str">
-        <x:v>Total after quantity change</x:v>
+        <x:v>Cart total after quantity change</x:v>
       </x:c>
       <x:c r="F65" s="14" t="str">
-        <x:v>Cart has item</x:v>
+        <x:v>Cart contains an item with quantity 2</x:v>
       </x:c>
       <x:c r="G65" s="14" t="str">
-        <x:v>₹250 ×2→×3</x:v>
+        <x:v>₹250 item; quantity 2→3</x:v>
       </x:c>
       <x:c r="H65" s="14" t="str">
-        <x:v>Change quantity; verify totals</x:v>
+        <x:v>Note current subtotal; increase quantity from 2 to 3; verify subtotal and applicable charges</x:v>
       </x:c>
       <x:c r="I65" s="14" t="str">
-        <x:v>Subtotal and charges recalculate</x:v>
+        <x:v>Subtotal and applicable charges are recalculated correctly after the quantity change</x:v>
       </x:c>
       <x:c r="J65" s="14" t="str">
         <x:v>High</x:v>
@@ -2405,19 +2406,19 @@
         <x:v>Coupon</x:v>
       </x:c>
       <x:c r="E66" s="14" t="str">
-        <x:v>Remove coupon and discount</x:v>
+        <x:v>Remove coupon and restore payable amount</x:v>
       </x:c>
       <x:c r="F66" s="14" t="str">
-        <x:v>Coupon applied</x:v>
+        <x:v>Eligible coupon is already applied</x:v>
       </x:c>
       <x:c r="G66" s="14" t="str">
         <x:v>WELCOME50</x:v>
       </x:c>
       <x:c r="H66" s="14" t="str">
-        <x:v>Remove coupon</x:v>
+        <x:v>Note discounted total; remove WELCOME50; verify discount and payable amount</x:v>
       </x:c>
       <x:c r="I66" s="14" t="str">
-        <x:v>Discount is removed and total restored</x:v>
+        <x:v>Coupon discount is removed and the applicable original payable amount is restored</x:v>
       </x:c>
       <x:c r="J66" s="14" t="str">
         <x:v>High</x:v>
@@ -2440,16 +2441,16 @@
         <x:v>Payment amount matches checkout</x:v>
       </x:c>
       <x:c r="F67" s="14" t="str">
-        <x:v>Checkout completed</x:v>
+        <x:v>Checkout is completed and final amount is available</x:v>
       </x:c>
       <x:c r="G67" s="14" t="str">
         <x:v>Checkout total ₹620</x:v>
       </x:c>
       <x:c r="H67" s="14" t="str">
-        <x:v>Compare checkout and payment amount</x:v>
+        <x:v>Note final checkout amount; proceed to Payment; compare the amount shown</x:v>
       </x:c>
       <x:c r="I67" s="14" t="str">
-        <x:v>Payment amount exactly matches checkout</x:v>
+        <x:v>Payment page amount exactly matches the final checkout payable amount</x:v>
       </x:c>
       <x:c r="J67" s="14" t="str">
         <x:v>High</x:v>
@@ -2472,16 +2473,16 @@
         <x:v>Complete food ordering journey</x:v>
       </x:c>
       <x:c r="F68" s="14" t="str">
-        <x:v>Application available</x:v>
+        <x:v>Application is available and required test data exists</x:v>
       </x:c>
       <x:c r="G68" s="14" t="str">
-        <x:v>New user; food; address; coupon; payment</x:v>
+        <x:v>New user; food item; address; eligible coupon; valid test payment</x:v>
       </x:c>
       <x:c r="H68" s="14" t="str">
-        <x:v>Register; login; search; cart; coupon; checkout; pay; order; track</x:v>
+        <x:v>Register; log in; search; add item; update cart; apply coupon; checkout; select address; pay; verify order; track order</x:v>
       </x:c>
       <x:c r="I68" s="14" t="str">
-        <x:v>Complete journey succeeds with consistent data</x:v>
+        <x:v>Complete user journey succeeds and order details remain consistent from checkout through tracking</x:v>
       </x:c>
       <x:c r="J68" s="14" t="str">
         <x:v>High</x:v>
@@ -2490,7 +2491,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R660c6d5670d142d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21592d490ebd4f3b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>